<commit_message>
feat: Lien ket nghiep vu xuyen suot trong cung 1 de thi va hoan thien tao de moi
</commit_message>
<xml_diff>
--- a/data/catalogs/patients.xlsx
+++ b/data/catalogs/patients.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1073,6 +1073,192 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>26030001</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Trần Văn An</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>15/03/1993</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Tân Lợi, Buôn Ma Thuột, Đắk Lắk</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>26030002</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Lê Thị Bình</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>20/05/1995</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Tân Lập, Buôn Ma Thuột, Đắk Lắk</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>26030003</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Phạm Văn Cường</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>12/08/1989</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Tự An, Buôn Ma Thuột, Đắk Lắk</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>26030004</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Hoàng Thị Dung</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>08/11/1992</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Tân An, Buôn Ma Thuột, Đắk Lắk</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>26030005</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Vũ Văn Giang</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>25/01/1987</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Ea Tam, Buôn Ma Thuột, Đắk Lắk</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>26030006</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Đặng Thị Hoa</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>30/04/1996</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Khánh Xuân, Buôn Ma Thuột, Đắk Lắk</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>